<commit_message>
[feat/HD-15488-BangladeshAdd-new-widget-non-functional-Disable-do-not-use-module-in-home-page] Replace formula with placeholder in the 'Do not use modules' report
</commit_message>
<xml_diff>
--- a/api/templates/do_not_use_modules_report/en.xlsx
+++ b/api/templates/do_not_use_modules_report/en.xlsx
@@ -9,7 +9,7 @@
     <sheet name="DisabledModules" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DisabledModules!$A$8:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DisabledModules!$A$8:$G$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DisabledModules!$A$8:$G$8</definedName>
   </definedNames>
   <calcPr/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">Disabled Modules</t>
   </si>
@@ -29,6 +29,9 @@
   </si>
   <si>
     <t xml:space="preserve">Count of Distinct Disabled Modules:</t>
+  </si>
+  <si>
+    <t>&lt;countOfDistinctDisabledModules&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;LgasLabel&gt;: &lt;Lgas&gt;</t>
@@ -736,72 +739,71 @@
       <c r="E3" t="s">
         <v>2</v>
       </c>
-      <c r="F3">
-        <f>IF(COUNTA(D9:D100000)=0,0,SUM(1/COUNTIF(D9:D100000,D9:D100000)))</f>
-        <v>1</v>
+      <c r="F3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" ht="16.5">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" ht="16.5">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" ht="16.5">
       <c r="A8" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="16.5">
       <c r="A9" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>